<commit_message>
Sheet | Effect 表目標類型/觸發時機欄位改名為 TargetKind/TriggerKind
更新 gamedata/Effect.xlsx 欄位英文名 TargetType→TargetKind、
TriggerType→TriggerKind，與 cores 列舉 Kind 命名一致；
sheeter 重新生成 sheet/effectReader.go 對應欄位。
效果類型欄位字面名為 Type，維持不變。

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gamedata/Effect.xlsx
+++ b/gamedata/Effect.xlsx
@@ -9,7 +9,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="t84dSBWrkW3C/+lLDhIF9Xi2tUEWC2dZty9iK1lGcaE="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="59IOp6KhDm3KXZvsqDvRn1+PuQA0GC6qcd/1ho7IHmQ="/>
     </ext>
   </extLst>
 </workbook>
@@ -78,7 +78,7 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mhVoOb6IlTNKXe1PkyX7S4ojGDFNw=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mjwAogtg0D84JMjd1t/0bj+G6S9Gw=="/>
     </ext>
   </extLst>
 </comments>
@@ -111,13 +111,13 @@
     <t>Group</t>
   </si>
   <si>
-    <t>TargetType</t>
+    <t>TargetKind</t>
   </si>
   <si>
     <t>TargetCount</t>
   </si>
   <si>
-    <t>TriggerType</t>
+    <t>TriggerKind</t>
   </si>
   <si>
     <t>TriggerCond</t>
@@ -247,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -256,6 +256,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -636,13 +639,13 @@
       <c r="E3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="3" t="s">
         <v>8</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I3" s="1" t="s">

</xml_diff>